<commit_message>
current mtech photos update and justify of home content
</commit_message>
<xml_diff>
--- a/excels/Current_Mtech.xlsx
+++ b/excels/Current_Mtech.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CED TD-11\Downloads\mainnn\NITW-Transportation-Division-main\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8418D07-C743-4968-8580-BA891E12D14F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180"/>
   </bookViews>
   <sheets>
     <sheet name="2024" sheetId="1" r:id="rId1"/>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="277">
   <si>
     <t>Name</t>
   </si>
@@ -620,6 +619,138 @@
   </si>
   <si>
     <t>Abhijit Namdeo Antarkar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thelu Venkata Sai Kumar </t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R02</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R03</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R05</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R06</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R08</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R09</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R10</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R11</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R12</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R13</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R14</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R15</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R16</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R17</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R18</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R19</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R20</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R21</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R22</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R23</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R24</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R25</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R26</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R27</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R28</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R29</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R30</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R31</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R32</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R39</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R40</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3S01</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3S02</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3S03</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3S04</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3S05</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3S06</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3S07</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3S08</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3S09</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3S10</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/25CEM3R07</t>
+  </si>
+  <si>
+    <t>Mtech_Current/2025/24CEM3S04</t>
   </si>
   <si>
     <t>Mtech_Current/2024/24CEM3R01</t>
@@ -730,8 +861,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -763,13 +894,6 @@
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -805,26 +929,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1104,15 +1228,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H43"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="41.85546875" customWidth="1"/>
-    <col min="3" max="3" width="121.85546875" customWidth="1"/>
-    <col min="7" max="7" width="28.85546875" customWidth="1"/>
-    <col min="8" max="8" width="29.85546875" style="10" customWidth="1"/>
+    <col min="1" max="1" width="26" style="5" customWidth="1"/>
+    <col min="2" max="2" width="41.85546875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="121.85546875" style="5" customWidth="1"/>
+    <col min="4" max="6" width="12.5703125" style="5"/>
+    <col min="7" max="7" width="28.85546875" style="5" customWidth="1"/>
+    <col min="8" max="8" width="29.85546875" style="11" customWidth="1"/>
+    <col min="9" max="16384" width="12.5703125" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1142,690 +1268,690 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>69</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="9" t="s">
-        <v>198</v>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="12" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>70</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="9" t="s">
-        <v>199</v>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="12" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>71</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="9" t="s">
-        <v>200</v>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="12" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>72</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="9" t="s">
-        <v>201</v>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="12" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>73</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="9" t="s">
-        <v>202</v>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="12" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>74</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="9" t="s">
-        <v>203</v>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="12" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>75</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="9" t="s">
-        <v>204</v>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="12" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>76</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="9" t="s">
-        <v>205</v>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="12" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>77</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="9" t="s">
-        <v>206</v>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="12" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="9" t="s">
-        <v>207</v>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="12" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>79</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="9" t="s">
-        <v>208</v>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="12" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="6" t="s">
         <v>80</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="9" t="s">
-        <v>209</v>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="12" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="6" t="s">
         <v>81</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="9" t="s">
-        <v>210</v>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="12" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>82</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="9" t="s">
-        <v>211</v>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="12" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="6" t="s">
         <v>83</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="9" t="s">
-        <v>212</v>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="12" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="6" t="s">
         <v>84</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="9" t="s">
-        <v>213</v>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="12" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="6" t="s">
         <v>85</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="9" t="s">
-        <v>214</v>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="12" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="6" t="s">
         <v>86</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="9" t="s">
-        <v>215</v>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="12" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="6" t="s">
         <v>87</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="9" t="s">
-        <v>216</v>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="12" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="6" t="s">
         <v>88</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="9" t="s">
-        <v>217</v>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="12" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="6" t="s">
         <v>89</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="9" t="s">
-        <v>218</v>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="12" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="6" t="s">
         <v>90</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="9" t="s">
-        <v>219</v>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="12" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="6" t="s">
         <v>91</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="9" t="s">
-        <v>220</v>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="12" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A25" s="5" t="s">
+      <c r="A25" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="6" t="s">
         <v>92</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="9" t="s">
-        <v>221</v>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="12" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="6" t="s">
         <v>93</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="9" t="s">
-        <v>222</v>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="12" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="6" t="s">
         <v>94</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="9" t="s">
-        <v>223</v>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="12" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A28" s="5" t="s">
+      <c r="A28" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="6" t="s">
         <v>95</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="D28" s="6"/>
-      <c r="E28" s="6"/>
-      <c r="F28" s="6"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="9" t="s">
-        <v>224</v>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="12" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="6" t="s">
         <v>96</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="D29" s="6"/>
-      <c r="E29" s="6"/>
-      <c r="F29" s="6"/>
-      <c r="G29" s="6"/>
-      <c r="H29" s="9" t="s">
-        <v>225</v>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="12" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A30" s="5" t="s">
+      <c r="A30" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="6" t="s">
         <v>97</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="9" t="s">
-        <v>226</v>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="8"/>
+      <c r="H30" s="12" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="6" t="s">
         <v>99</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="9" t="s">
-        <v>227</v>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="12" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
+      <c r="A32" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
-      <c r="H32" s="9" t="s">
-        <v>228</v>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="12" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
+      <c r="A33" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" s="7" t="s">
         <v>103</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="6"/>
-      <c r="G33" s="6"/>
-      <c r="H33" s="9" t="s">
-        <v>229</v>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="12" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
+      <c r="A34" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="7" t="s">
         <v>105</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D34" s="6"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
-      <c r="H34" s="9" t="s">
-        <v>230</v>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="8"/>
+      <c r="H34" s="12" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
+      <c r="A35" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" s="7" t="s">
         <v>107</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="D35" s="6"/>
-      <c r="E35" s="6"/>
-      <c r="F35" s="6"/>
-      <c r="G35" s="6"/>
-      <c r="H35" s="9" t="s">
-        <v>231</v>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="12" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
+      <c r="A36" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="7" t="s">
         <v>109</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="9" t="s">
-        <v>232</v>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="12" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="1"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="7"/>
     </row>
     <row r="38" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="C38" s="6"/>
-      <c r="D38" s="6"/>
-      <c r="E38" s="6"/>
-      <c r="F38" s="6"/>
-      <c r="G38" s="6"/>
-      <c r="H38" s="1"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C39" s="9"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="9"/>
-      <c r="G39" s="9"/>
-      <c r="H39" s="5"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8"/>
+      <c r="H38" s="7"/>
+    </row>
+    <row r="39" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C40" s="9"/>
-      <c r="D40" s="9"/>
-      <c r="E40" s="9"/>
-      <c r="F40" s="9"/>
-      <c r="G40" s="9"/>
-      <c r="H40" s="5"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="6"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C41" s="9"/>
-      <c r="D41" s="9"/>
-      <c r="E41" s="9"/>
-      <c r="F41" s="9"/>
-      <c r="G41" s="9"/>
-      <c r="H41" s="5"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="6"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C42" s="9"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="9"/>
-      <c r="F42" s="9"/>
-      <c r="G42" s="9"/>
-      <c r="H42" s="5"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="10"/>
+      <c r="F42" s="10"/>
+      <c r="G42" s="10"/>
+      <c r="H42" s="6"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C43" s="9"/>
-      <c r="D43" s="9"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="9"/>
-      <c r="G43" s="9"/>
-      <c r="H43" s="5"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1833,7 +1959,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1844,6 +1970,7 @@
     <col min="5" max="5" width="26.5703125" customWidth="1"/>
     <col min="6" max="6" width="28" customWidth="1"/>
     <col min="7" max="7" width="29.85546875" customWidth="1"/>
+    <col min="8" max="8" width="38.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
@@ -1873,434 +2000,692 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="H2" s="8"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="H3" s="8"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="H4" s="8"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="H5" s="8"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="H6" s="8"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="H7" s="8"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="H8" s="8"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" t="s">
+        <v>204</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="H9" s="8"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="H10" s="8"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" t="s">
+        <v>206</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="H11" s="8"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" t="s">
+        <v>207</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="H12" s="8"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" t="s">
+        <v>208</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="C13" s="7"/>
-      <c r="H13" s="8"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="C14" s="7"/>
-      <c r="H14" s="8"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="C15" s="7"/>
-      <c r="H15" s="8"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" t="s">
+        <v>211</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="C16" s="7"/>
-      <c r="H16" s="8"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" t="s">
+        <v>212</v>
+      </c>
     </row>
     <row r="17" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="H17" s="8"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" t="s">
+        <v>213</v>
+      </c>
     </row>
     <row r="18" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="H18" s="8"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" t="s">
+        <v>214</v>
+      </c>
     </row>
     <row r="19" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="C19" s="7"/>
-      <c r="H19" s="8"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" t="s">
+        <v>215</v>
+      </c>
     </row>
     <row r="20" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="C20" s="7"/>
-      <c r="H20" s="8"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" t="s">
+        <v>216</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="C21" s="7"/>
-      <c r="H21" s="8"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="22" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="C22" s="7"/>
-      <c r="H22" s="8"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" t="s">
+        <v>218</v>
+      </c>
     </row>
     <row r="23" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="C23" s="7"/>
-      <c r="H23" s="8"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="24" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="C24" s="7"/>
-      <c r="H24" s="8"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="25" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
+      <c r="A25" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="C25" s="7"/>
-      <c r="H25" s="8"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="26" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="H26" s="8"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" t="s">
+        <v>222</v>
+      </c>
     </row>
     <row r="27" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="C27" s="7"/>
-      <c r="H27" s="8"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" t="s">
+        <v>223</v>
+      </c>
     </row>
     <row r="28" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="5" t="s">
+      <c r="A28" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C28" s="9"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+      <c r="H28" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="C28" s="7"/>
-      <c r="H28" s="8"/>
-    </row>
-    <row r="29" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="C29" s="7"/>
-      <c r="H29" s="8"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="30" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="5" t="s">
+      <c r="A30" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="C30" s="7"/>
-      <c r="H30" s="8"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+      <c r="G30" s="5"/>
+      <c r="H30" t="s">
+        <v>226</v>
+      </c>
     </row>
     <row r="31" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="C31" s="7"/>
-      <c r="H31" s="8"/>
+      <c r="C31" s="9"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" t="s">
+        <v>227</v>
+      </c>
     </row>
     <row r="32" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="5" t="s">
+      <c r="A32" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="C32" s="7"/>
-      <c r="H32" s="8"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="33" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="5" t="s">
+      <c r="A33" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B33" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="C33" s="7"/>
-      <c r="H33" s="8"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" t="s">
+        <v>229</v>
+      </c>
     </row>
     <row r="34" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="5" t="s">
+      <c r="A34" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="C34" s="7"/>
-      <c r="H34" s="8"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="35" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="5" t="s">
+      <c r="A35" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="C35" s="7"/>
-      <c r="H35" s="8"/>
+      <c r="C35" s="9"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" t="s">
+        <v>231</v>
+      </c>
     </row>
     <row r="36" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="5" t="s">
+      <c r="A36" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="C36" s="7"/>
-      <c r="H36" s="8"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="37" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A37" s="5" t="s">
+      <c r="A37" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="C37" s="7"/>
-      <c r="H37" s="8"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+      <c r="H37" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="38" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A38" s="5" t="s">
+      <c r="A38" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="B38" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="C38" s="7"/>
-      <c r="H38" s="8"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="5"/>
+      <c r="H38" t="s">
+        <v>241</v>
+      </c>
     </row>
     <row r="39" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A39" s="5" t="s">
+      <c r="A39" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="B39" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="C39" s="7"/>
-      <c r="H39" s="8"/>
+      <c r="C39" s="9"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="5"/>
+      <c r="F39" s="5"/>
+      <c r="G39" s="5"/>
+      <c r="H39" t="s">
+        <v>234</v>
+      </c>
     </row>
     <row r="40" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A40" s="5" t="s">
+      <c r="A40" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="B40" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="C40" s="7"/>
-      <c r="H40" s="8"/>
+      <c r="C40" s="9"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+      <c r="H40" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="41" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A41" s="5" t="s">
+      <c r="A41" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="B41" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="C41" s="7"/>
-      <c r="H41" s="8"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" t="s">
+        <v>236</v>
+      </c>
     </row>
     <row r="42" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="B42" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="C42" s="7"/>
-      <c r="H42" s="8"/>
+      <c r="C42" s="9"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="5"/>
+      <c r="H42" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="43" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A43" s="5" t="s">
+      <c r="A43" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="B43" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="C43" s="7"/>
-      <c r="H43" s="8"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="5"/>
+      <c r="E43" s="5"/>
+      <c r="F43" s="5"/>
+      <c r="G43" s="5"/>
+      <c r="H43" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="44" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A44" s="5" t="s">
+      <c r="A44" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="B44" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="C44" s="7"/>
-      <c r="H44" s="8"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
+      <c r="H44" t="s">
+        <v>239</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated PHD Thesis abstract pop and nitw LOGO
</commit_message>
<xml_diff>
--- a/excels/Current_Mtech.xlsx
+++ b/excels/Current_Mtech.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="2024" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="276">
   <si>
     <t>Name</t>
   </si>
@@ -229,9 +229,6 @@
   </si>
   <si>
     <t xml:space="preserve">Industry Training </t>
-  </si>
-  <si>
-    <t>Current Position</t>
   </si>
   <si>
     <t>Dhanavath Ajay</t>
@@ -1229,19 +1226,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" style="5" customWidth="1"/>
     <col min="2" max="2" width="41.85546875" style="5" customWidth="1"/>
     <col min="3" max="3" width="121.85546875" style="5" customWidth="1"/>
     <col min="4" max="6" width="12.5703125" style="5"/>
-    <col min="7" max="7" width="28.85546875" style="5" customWidth="1"/>
-    <col min="8" max="8" width="29.85546875" style="11" customWidth="1"/>
-    <col min="9" max="16384" width="12.5703125" style="5"/>
+    <col min="7" max="7" width="29.85546875" style="11" customWidth="1"/>
+    <col min="8" max="16384" width="12.5703125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>64</v>
       </c>
@@ -1260,698 +1256,653 @@
       <c r="F1" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="H1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>35</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
       <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="12" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G2" s="12" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>36</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
       <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="12" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G3" s="12" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>37</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
       <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="12" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G4" s="12" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>38</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
       <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="12" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G5" s="12" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>39</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D6" s="8"/>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="12" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G6" s="12" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>40</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="12" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G7" s="12" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>41</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="12" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G8" s="12" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>42</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D9" s="8"/>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="12" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G9" s="12" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>43</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D10" s="8"/>
       <c r="E10" s="8"/>
       <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="12" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G10" s="12" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>44</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D11" s="8"/>
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="12" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G11" s="12" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>45</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="12" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G12" s="12" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>46</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="12" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G13" s="12" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>47</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="12" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G14" s="12" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>48</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
       <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="12" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G15" s="12" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>49</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="12" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G16" s="12" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>50</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
       <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="12" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G17" s="12" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>51</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
       <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="12" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G18" s="12" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
         <v>52</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D19" s="8"/>
       <c r="E19" s="8"/>
       <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="12" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G19" s="12" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>53</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D20" s="8"/>
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="12" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G20" s="12" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>54</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D21" s="8"/>
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="12" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G21" s="12" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>55</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="12" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G22" s="12" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>56</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D23" s="8"/>
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="12" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G23" s="12" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>57</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D24" s="8"/>
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="12" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G24" s="12" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>58</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="12" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G25" s="12" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
         <v>59</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D26" s="8"/>
       <c r="E26" s="8"/>
       <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="12" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G26" s="12" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
         <v>60</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D27" s="8"/>
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="12" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G27" s="12" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
         <v>61</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D28" s="8"/>
       <c r="E28" s="8"/>
       <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="12" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G28" s="12" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
         <v>62</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D29" s="8"/>
       <c r="E29" s="8"/>
       <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="12" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G29" s="12" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
         <v>63</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D30" s="8"/>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="12" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G30" s="12" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B31" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="B31" s="6" t="s">
-        <v>99</v>
-      </c>
       <c r="C31" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D31" s="8"/>
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
-      <c r="G31" s="8"/>
-      <c r="H31" s="12" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G31" s="12" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B32" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="B32" s="7" t="s">
-        <v>101</v>
-      </c>
       <c r="C32" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D32" s="8"/>
       <c r="E32" s="8"/>
       <c r="F32" s="8"/>
-      <c r="G32" s="8"/>
-      <c r="H32" s="12" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G32" s="12" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B33" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="B33" s="7" t="s">
-        <v>103</v>
-      </c>
       <c r="C33" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D33" s="8"/>
       <c r="E33" s="8"/>
       <c r="F33" s="8"/>
-      <c r="G33" s="8"/>
-      <c r="H33" s="12" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G33" s="12" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B34" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="B34" s="7" t="s">
-        <v>105</v>
-      </c>
       <c r="C34" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D34" s="8"/>
       <c r="E34" s="8"/>
       <c r="F34" s="8"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="12" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G34" s="12" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A35" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B35" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B35" s="7" t="s">
-        <v>107</v>
-      </c>
       <c r="C35" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D35" s="8"/>
       <c r="E35" s="8"/>
       <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="12" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G35" s="12" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="B36" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="B36" s="7" t="s">
-        <v>109</v>
-      </c>
       <c r="C36" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D36" s="8"/>
       <c r="E36" s="8"/>
       <c r="F36" s="8"/>
-      <c r="G36" s="8"/>
-      <c r="H36" s="12" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G36" s="12" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="C37" s="8"/>
       <c r="D37" s="8"/>
       <c r="E37" s="8"/>
       <c r="F37" s="8"/>
-      <c r="G37" s="8"/>
-      <c r="H37" s="7"/>
-    </row>
-    <row r="38" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G37" s="7"/>
+    </row>
+    <row r="38" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="C38" s="8"/>
       <c r="D38" s="8"/>
       <c r="E38" s="8"/>
       <c r="F38" s="8"/>
-      <c r="G38" s="8"/>
-      <c r="H38" s="7"/>
-    </row>
-    <row r="39" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="G38" s="7"/>
+    </row>
+    <row r="39" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="C39" s="10"/>
       <c r="D39" s="10"/>
       <c r="E39" s="10"/>
       <c r="F39" s="10"/>
       <c r="G39" s="10"/>
-      <c r="H39" s="10"/>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C40" s="10"/>
       <c r="D40" s="10"/>
       <c r="E40" s="10"/>
       <c r="F40" s="10"/>
-      <c r="G40" s="10"/>
-      <c r="H40" s="6"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G40" s="6"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C41" s="10"/>
       <c r="D41" s="10"/>
       <c r="E41" s="10"/>
       <c r="F41" s="10"/>
-      <c r="G41" s="10"/>
-      <c r="H41" s="6"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G41" s="6"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C42" s="10"/>
       <c r="D42" s="10"/>
       <c r="E42" s="10"/>
       <c r="F42" s="10"/>
-      <c r="G42" s="10"/>
-      <c r="H42" s="6"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G42" s="6"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C43" s="10"/>
       <c r="D43" s="10"/>
       <c r="E43" s="10"/>
       <c r="F43" s="10"/>
-      <c r="G43" s="10"/>
-      <c r="H43" s="6"/>
+      <c r="G43" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1960,7 +1911,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -1969,11 +1920,10 @@
     <col min="4" max="4" width="19.28515625" customWidth="1"/>
     <col min="5" max="5" width="26.5703125" customWidth="1"/>
     <col min="6" max="6" width="28" customWidth="1"/>
-    <col min="7" max="7" width="29.85546875" customWidth="1"/>
-    <col min="8" max="8" width="38.28515625" customWidth="1"/>
+    <col min="7" max="7" width="38.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>64</v>
       </c>
@@ -1992,699 +1942,653 @@
       <c r="F1" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="H1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C2" s="9"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C3" s="9"/>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
       <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G3" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C4" s="9"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G5" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C6" s="9"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G6" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G7" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C8" s="9"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G8" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C9" s="9"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G9" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>11</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C10" s="9"/>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G10" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>12</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C11" s="9"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G11" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>13</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C12" s="9"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G12" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>14</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C13" s="9"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G13" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C14" s="9"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G14" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>16</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C15" s="9"/>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
       <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G15" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C16" s="9"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G16" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>18</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G17" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>19</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C18" s="9"/>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G18" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>20</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G19" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>21</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C20" s="9"/>
       <c r="D20" s="5"/>
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G20" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C21" s="9"/>
       <c r="D21" s="5"/>
       <c r="E21" s="5"/>
       <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G21" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C22" s="9"/>
       <c r="D22" s="5"/>
       <c r="E22" s="5"/>
       <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G22" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>24</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C23" s="9"/>
       <c r="D23" s="5"/>
       <c r="E23" s="5"/>
       <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G23" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>25</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C24" s="9"/>
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
       <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G24" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C25" s="9"/>
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
       <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
-      <c r="H25" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G25" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>27</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C26" s="9"/>
       <c r="D26" s="5"/>
       <c r="E26" s="5"/>
       <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
-      <c r="H26" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G26" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>28</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C27" s="9"/>
       <c r="D27" s="5"/>
       <c r="E27" s="5"/>
       <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
-      <c r="H27" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G27" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>29</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C28" s="9"/>
       <c r="D28" s="5"/>
       <c r="E28" s="5"/>
       <c r="F28" s="5"/>
-      <c r="G28" s="5"/>
-      <c r="H28" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G28" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>30</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C29" s="9"/>
       <c r="D29" s="5"/>
       <c r="E29" s="5"/>
       <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
-      <c r="H29" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G29" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C30" s="9"/>
       <c r="D30" s="5"/>
       <c r="E30" s="5"/>
       <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
-      <c r="H30" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G30" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>32</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C31" s="9"/>
       <c r="D31" s="5"/>
       <c r="E31" s="5"/>
       <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
-      <c r="H31" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G31" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>33</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C32" s="9"/>
       <c r="D32" s="5"/>
       <c r="E32" s="5"/>
       <c r="F32" s="5"/>
-      <c r="G32" s="5"/>
-      <c r="H32" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G32" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>34</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C33" s="9"/>
       <c r="D33" s="5"/>
       <c r="E33" s="5"/>
       <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
-      <c r="H33" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G33" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C34" s="9"/>
       <c r="D34" s="5"/>
       <c r="E34" s="5"/>
       <c r="F34" s="5"/>
-      <c r="G34" s="5"/>
-      <c r="H34" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G34" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C35" s="9"/>
       <c r="D35" s="5"/>
       <c r="E35" s="5"/>
       <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-      <c r="H35" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G35" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C36" s="9"/>
       <c r="D36" s="5"/>
       <c r="E36" s="5"/>
       <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
-      <c r="H36" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G36" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C37" s="9"/>
       <c r="D37" s="5"/>
       <c r="E37" s="5"/>
       <c r="F37" s="5"/>
-      <c r="G37" s="5"/>
-      <c r="H37" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G37" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="B38" s="6" t="s">
         <v>191</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>192</v>
       </c>
       <c r="C38" s="9"/>
       <c r="D38" s="5"/>
       <c r="E38" s="5"/>
       <c r="F38" s="5"/>
-      <c r="G38" s="5"/>
-      <c r="H38" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G38" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="B39" s="6" t="s">
         <v>150</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>151</v>
       </c>
       <c r="C39" s="9"/>
       <c r="D39" s="5"/>
       <c r="E39" s="5"/>
       <c r="F39" s="5"/>
-      <c r="G39" s="5"/>
-      <c r="H39" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G39" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C40" s="9"/>
       <c r="D40" s="5"/>
       <c r="E40" s="5"/>
       <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
-      <c r="H40" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G40" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C41" s="9"/>
       <c r="D41" s="5"/>
       <c r="E41" s="5"/>
       <c r="F41" s="5"/>
-      <c r="G41" s="5"/>
-      <c r="H41" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G41" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C42" s="9"/>
       <c r="D42" s="5"/>
       <c r="E42" s="5"/>
       <c r="F42" s="5"/>
-      <c r="G42" s="5"/>
-      <c r="H42" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G42" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C43" s="9"/>
       <c r="D43" s="5"/>
       <c r="E43" s="5"/>
       <c r="F43" s="5"/>
-      <c r="G43" s="5"/>
-      <c r="H43" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G43" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C44" s="9"/>
       <c r="D44" s="5"/>
       <c r="E44" s="5"/>
       <c r="F44" s="5"/>
-      <c r="G44" s="5"/>
-      <c r="H44" t="s">
-        <v>239</v>
+      <c r="G44" t="s">
+        <v>238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated supervisor in mtech current
</commit_message>
<xml_diff>
--- a/excels/Current_Mtech.xlsx
+++ b/excels/Current_Mtech.xlsx
@@ -15,6 +15,9 @@
     <sheet name="2024" sheetId="1" r:id="rId1"/>
     <sheet name="2025" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2025'!$E$1:$E$44</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -25,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="285">
   <si>
     <t>Name</t>
   </si>
@@ -504,9 +507,6 @@
     <t>AYUSHA ARUN BHAMARE</t>
   </si>
   <si>
-    <t>Babu Kumar Patel</t>
-  </si>
-  <si>
     <t>B. Datta Vamsi</t>
   </si>
   <si>
@@ -853,13 +853,43 @@
   </si>
   <si>
     <t>Mtech_Current/2024/24CEM3S06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supervisor and Co-Supervisor </t>
+  </si>
+  <si>
+    <t>Prof. Arpan Mehar</t>
+  </si>
+  <si>
+    <t>Prof. Venkaiah Chowdary</t>
+  </si>
+  <si>
+    <t>Prof. S. Shankar</t>
+  </si>
+  <si>
+    <t>Prof. Vishnu R.</t>
+  </si>
+  <si>
+    <t>Prof. Bhadradri Raghuram Kadali</t>
+  </si>
+  <si>
+    <t>Prof. K.V.R. Ravi Shankar</t>
+  </si>
+  <si>
+    <t>Seminar Abstract</t>
+  </si>
+  <si>
+    <t>Supervisor and Co-Supervisor</t>
+  </si>
+  <si>
+    <t>Bablu Kumar Patel</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -905,6 +935,18 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman "/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -926,7 +968,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -946,6 +988,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1226,18 +1274,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G43"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H43"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="26" style="5" customWidth="1"/>
     <col min="2" max="2" width="41.85546875" style="5" customWidth="1"/>
     <col min="3" max="3" width="121.85546875" style="5" customWidth="1"/>
-    <col min="4" max="6" width="12.5703125" style="5"/>
-    <col min="7" max="7" width="29.85546875" style="11" customWidth="1"/>
-    <col min="8" max="16384" width="12.5703125" style="5"/>
+    <col min="4" max="4" width="12.5703125" style="5"/>
+    <col min="5" max="5" width="52.7109375" style="16" customWidth="1"/>
+    <col min="6" max="7" width="12.5703125" style="5"/>
+    <col min="8" max="8" width="29.85546875" style="11" customWidth="1"/>
+    <col min="9" max="16384" width="12.5703125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="15.75" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>64</v>
       </c>
@@ -1250,17 +1300,20 @@
       <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="13" t="s">
+        <v>275</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18.75">
       <c r="A2" s="6" t="s">
         <v>35</v>
       </c>
@@ -1271,13 +1324,16 @@
         <v>109</v>
       </c>
       <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
+      <c r="E2" s="14" t="s">
+        <v>276</v>
+      </c>
       <c r="F2" s="8"/>
-      <c r="G2" s="12" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G2" s="8"/>
+      <c r="H2" s="12" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="18.75">
       <c r="A3" s="6" t="s">
         <v>36</v>
       </c>
@@ -1288,13 +1344,16 @@
         <v>110</v>
       </c>
       <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
+      <c r="E3" s="14" t="s">
+        <v>277</v>
+      </c>
       <c r="F3" s="8"/>
-      <c r="G3" s="12" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G3" s="8"/>
+      <c r="H3" s="12" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="18.75">
       <c r="A4" s="6" t="s">
         <v>37</v>
       </c>
@@ -1305,13 +1364,16 @@
         <v>111</v>
       </c>
       <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
+      <c r="E4" s="14" t="s">
+        <v>277</v>
+      </c>
       <c r="F4" s="8"/>
-      <c r="G4" s="12" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G4" s="8"/>
+      <c r="H4" s="12" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="18.75">
       <c r="A5" s="6" t="s">
         <v>38</v>
       </c>
@@ -1322,13 +1384,16 @@
         <v>112</v>
       </c>
       <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
+      <c r="E5" s="14" t="s">
+        <v>278</v>
+      </c>
       <c r="F5" s="8"/>
-      <c r="G5" s="12" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G5" s="8"/>
+      <c r="H5" s="12" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="18.75">
       <c r="A6" s="6" t="s">
         <v>39</v>
       </c>
@@ -1339,13 +1404,16 @@
         <v>113</v>
       </c>
       <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
+      <c r="E6" s="14" t="s">
+        <v>276</v>
+      </c>
       <c r="F6" s="8"/>
-      <c r="G6" s="12" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G6" s="8"/>
+      <c r="H6" s="12" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="18.75">
       <c r="A7" s="6" t="s">
         <v>40</v>
       </c>
@@ -1356,13 +1424,16 @@
         <v>114</v>
       </c>
       <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
+      <c r="E7" s="14" t="s">
+        <v>279</v>
+      </c>
       <c r="F7" s="8"/>
-      <c r="G7" s="12" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G7" s="8"/>
+      <c r="H7" s="12" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="18.75">
       <c r="A8" s="6" t="s">
         <v>41</v>
       </c>
@@ -1373,13 +1444,16 @@
         <v>115</v>
       </c>
       <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
+      <c r="E8" s="14" t="s">
+        <v>277</v>
+      </c>
       <c r="F8" s="8"/>
-      <c r="G8" s="12" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G8" s="8"/>
+      <c r="H8" s="12" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="18.75">
       <c r="A9" s="6" t="s">
         <v>42</v>
       </c>
@@ -1390,13 +1464,16 @@
         <v>116</v>
       </c>
       <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
+      <c r="E9" s="15" t="s">
+        <v>280</v>
+      </c>
       <c r="F9" s="8"/>
-      <c r="G9" s="12" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G9" s="8"/>
+      <c r="H9" s="12" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="18.75">
       <c r="A10" s="6" t="s">
         <v>43</v>
       </c>
@@ -1407,13 +1484,16 @@
         <v>117</v>
       </c>
       <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
+      <c r="E10" s="14" t="s">
+        <v>277</v>
+      </c>
       <c r="F10" s="8"/>
-      <c r="G10" s="12" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G10" s="8"/>
+      <c r="H10" s="12" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="18.75">
       <c r="A11" s="6" t="s">
         <v>44</v>
       </c>
@@ -1424,13 +1504,16 @@
         <v>118</v>
       </c>
       <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
+      <c r="E11" s="15" t="s">
+        <v>280</v>
+      </c>
       <c r="F11" s="8"/>
-      <c r="G11" s="12" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G11" s="8"/>
+      <c r="H11" s="12" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="18.75">
       <c r="A12" s="6" t="s">
         <v>45</v>
       </c>
@@ -1441,13 +1524,16 @@
         <v>119</v>
       </c>
       <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
+      <c r="E12" s="14" t="s">
+        <v>276</v>
+      </c>
       <c r="F12" s="8"/>
-      <c r="G12" s="12" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G12" s="8"/>
+      <c r="H12" s="12" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="18.75">
       <c r="A13" s="6" t="s">
         <v>46</v>
       </c>
@@ -1458,13 +1544,16 @@
         <v>120</v>
       </c>
       <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
+      <c r="E13" s="14" t="s">
+        <v>281</v>
+      </c>
       <c r="F13" s="8"/>
-      <c r="G13" s="12" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G13" s="8"/>
+      <c r="H13" s="12" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="18.75">
       <c r="A14" s="6" t="s">
         <v>47</v>
       </c>
@@ -1475,13 +1564,16 @@
         <v>121</v>
       </c>
       <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
+      <c r="E14" s="14" t="s">
+        <v>277</v>
+      </c>
       <c r="F14" s="8"/>
-      <c r="G14" s="12" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G14" s="8"/>
+      <c r="H14" s="12" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="18.75">
       <c r="A15" s="6" t="s">
         <v>48</v>
       </c>
@@ -1492,13 +1584,16 @@
         <v>122</v>
       </c>
       <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
+      <c r="E15" s="15" t="s">
+        <v>280</v>
+      </c>
       <c r="F15" s="8"/>
-      <c r="G15" s="12" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G15" s="8"/>
+      <c r="H15" s="12" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="18.75">
       <c r="A16" s="6" t="s">
         <v>49</v>
       </c>
@@ -1509,13 +1604,16 @@
         <v>123</v>
       </c>
       <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
+      <c r="E16" s="14" t="s">
+        <v>277</v>
+      </c>
       <c r="F16" s="8"/>
-      <c r="G16" s="12" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G16" s="8"/>
+      <c r="H16" s="12" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="18.75">
       <c r="A17" s="6" t="s">
         <v>50</v>
       </c>
@@ -1526,13 +1624,16 @@
         <v>124</v>
       </c>
       <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
+      <c r="E17" s="14" t="s">
+        <v>276</v>
+      </c>
       <c r="F17" s="8"/>
-      <c r="G17" s="12" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G17" s="8"/>
+      <c r="H17" s="12" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="18.75">
       <c r="A18" s="6" t="s">
         <v>51</v>
       </c>
@@ -1543,13 +1644,16 @@
         <v>125</v>
       </c>
       <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
+      <c r="E18" s="14" t="s">
+        <v>276</v>
+      </c>
       <c r="F18" s="8"/>
-      <c r="G18" s="12" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G18" s="8"/>
+      <c r="H18" s="12" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="18.75">
       <c r="A19" s="6" t="s">
         <v>52</v>
       </c>
@@ -1560,13 +1664,16 @@
         <v>126</v>
       </c>
       <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
+      <c r="E19" s="14" t="s">
+        <v>279</v>
+      </c>
       <c r="F19" s="8"/>
-      <c r="G19" s="12" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G19" s="8"/>
+      <c r="H19" s="12" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="18.75">
       <c r="A20" s="6" t="s">
         <v>53</v>
       </c>
@@ -1577,13 +1684,16 @@
         <v>127</v>
       </c>
       <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
+      <c r="E20" s="15" t="s">
+        <v>280</v>
+      </c>
       <c r="F20" s="8"/>
-      <c r="G20" s="12" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G20" s="8"/>
+      <c r="H20" s="12" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="18.75">
       <c r="A21" s="6" t="s">
         <v>54</v>
       </c>
@@ -1594,13 +1704,16 @@
         <v>128</v>
       </c>
       <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
+      <c r="E21" s="14" t="s">
+        <v>279</v>
+      </c>
       <c r="F21" s="8"/>
-      <c r="G21" s="12" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G21" s="8"/>
+      <c r="H21" s="12" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="18.75">
       <c r="A22" s="6" t="s">
         <v>55</v>
       </c>
@@ -1611,13 +1724,16 @@
         <v>129</v>
       </c>
       <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
+      <c r="E22" s="14" t="s">
+        <v>279</v>
+      </c>
       <c r="F22" s="8"/>
-      <c r="G22" s="12" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G22" s="8"/>
+      <c r="H22" s="12" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="18.75">
       <c r="A23" s="6" t="s">
         <v>56</v>
       </c>
@@ -1628,13 +1744,16 @@
         <v>130</v>
       </c>
       <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
+      <c r="E23" s="14" t="s">
+        <v>278</v>
+      </c>
       <c r="F23" s="8"/>
-      <c r="G23" s="12" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G23" s="8"/>
+      <c r="H23" s="12" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="18.75">
       <c r="A24" s="6" t="s">
         <v>57</v>
       </c>
@@ -1645,13 +1764,16 @@
         <v>131</v>
       </c>
       <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
+      <c r="E24" s="14" t="s">
+        <v>281</v>
+      </c>
       <c r="F24" s="8"/>
-      <c r="G24" s="12" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G24" s="8"/>
+      <c r="H24" s="12" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="18.75">
       <c r="A25" s="6" t="s">
         <v>58</v>
       </c>
@@ -1662,13 +1784,16 @@
         <v>132</v>
       </c>
       <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
+      <c r="E25" s="14" t="s">
+        <v>278</v>
+      </c>
       <c r="F25" s="8"/>
-      <c r="G25" s="12" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G25" s="8"/>
+      <c r="H25" s="12" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="18.75">
       <c r="A26" s="6" t="s">
         <v>59</v>
       </c>
@@ -1679,13 +1804,16 @@
         <v>133</v>
       </c>
       <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
+      <c r="E26" s="14" t="s">
+        <v>281</v>
+      </c>
       <c r="F26" s="8"/>
-      <c r="G26" s="12" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G26" s="8"/>
+      <c r="H26" s="12" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="18.75">
       <c r="A27" s="6" t="s">
         <v>60</v>
       </c>
@@ -1696,13 +1824,16 @@
         <v>134</v>
       </c>
       <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
+      <c r="E27" s="14" t="s">
+        <v>279</v>
+      </c>
       <c r="F27" s="8"/>
-      <c r="G27" s="12" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G27" s="8"/>
+      <c r="H27" s="12" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="18.75">
       <c r="A28" s="6" t="s">
         <v>61</v>
       </c>
@@ -1713,13 +1844,16 @@
         <v>135</v>
       </c>
       <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
+      <c r="E28" s="14" t="s">
+        <v>281</v>
+      </c>
       <c r="F28" s="8"/>
-      <c r="G28" s="12" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G28" s="8"/>
+      <c r="H28" s="12" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="18.75">
       <c r="A29" s="6" t="s">
         <v>62</v>
       </c>
@@ -1730,13 +1864,16 @@
         <v>136</v>
       </c>
       <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
+      <c r="E29" s="14" t="s">
+        <v>276</v>
+      </c>
       <c r="F29" s="8"/>
-      <c r="G29" s="12" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G29" s="8"/>
+      <c r="H29" s="12" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="18.75">
       <c r="A30" s="6" t="s">
         <v>63</v>
       </c>
@@ -1747,13 +1884,16 @@
         <v>137</v>
       </c>
       <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
+      <c r="E30" s="14" t="s">
+        <v>281</v>
+      </c>
       <c r="F30" s="8"/>
-      <c r="G30" s="12" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G30" s="8"/>
+      <c r="H30" s="12" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="18.75">
       <c r="A31" s="6" t="s">
         <v>97</v>
       </c>
@@ -1764,13 +1904,16 @@
         <v>138</v>
       </c>
       <c r="D31" s="8"/>
-      <c r="E31" s="8"/>
+      <c r="E31" s="14" t="s">
+        <v>276</v>
+      </c>
       <c r="F31" s="8"/>
-      <c r="G31" s="12" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G31" s="8"/>
+      <c r="H31" s="12" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="18.75">
       <c r="A32" s="7" t="s">
         <v>99</v>
       </c>
@@ -1781,13 +1924,16 @@
         <v>139</v>
       </c>
       <c r="D32" s="8"/>
-      <c r="E32" s="8"/>
+      <c r="E32" s="14" t="s">
+        <v>278</v>
+      </c>
       <c r="F32" s="8"/>
-      <c r="G32" s="12" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G32" s="8"/>
+      <c r="H32" s="12" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="18.75">
       <c r="A33" s="7" t="s">
         <v>101</v>
       </c>
@@ -1798,13 +1944,16 @@
         <v>140</v>
       </c>
       <c r="D33" s="8"/>
-      <c r="E33" s="8"/>
+      <c r="E33" s="15" t="s">
+        <v>280</v>
+      </c>
       <c r="F33" s="8"/>
-      <c r="G33" s="12" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G33" s="8"/>
+      <c r="H33" s="12" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="18.75">
       <c r="A34" s="7" t="s">
         <v>103</v>
       </c>
@@ -1815,13 +1964,16 @@
         <v>141</v>
       </c>
       <c r="D34" s="8"/>
-      <c r="E34" s="8"/>
+      <c r="E34" s="15" t="s">
+        <v>280</v>
+      </c>
       <c r="F34" s="8"/>
-      <c r="G34" s="12" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G34" s="8"/>
+      <c r="H34" s="12" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="18.75">
       <c r="A35" s="7" t="s">
         <v>105</v>
       </c>
@@ -1832,13 +1984,16 @@
         <v>142</v>
       </c>
       <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
+      <c r="E35" s="15" t="s">
+        <v>280</v>
+      </c>
       <c r="F35" s="8"/>
-      <c r="G35" s="12" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G35" s="8"/>
+      <c r="H35" s="12" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="18.75">
       <c r="A36" s="7" t="s">
         <v>107</v>
       </c>
@@ -1849,60 +2004,63 @@
         <v>143</v>
       </c>
       <c r="D36" s="8"/>
-      <c r="E36" s="8"/>
+      <c r="E36" s="14" t="s">
+        <v>281</v>
+      </c>
       <c r="F36" s="8"/>
-      <c r="G36" s="12" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G36" s="8"/>
+      <c r="H36" s="12" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="18.75">
       <c r="C37" s="8"/>
       <c r="D37" s="8"/>
-      <c r="E37" s="8"/>
       <c r="F37" s="8"/>
-      <c r="G37" s="7"/>
-    </row>
-    <row r="38" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G37" s="8"/>
+      <c r="H37" s="7"/>
+    </row>
+    <row r="38" spans="1:8" ht="18.75">
       <c r="C38" s="8"/>
       <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
       <c r="F38" s="8"/>
-      <c r="G38" s="7"/>
-    </row>
-    <row r="39" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="G38" s="8"/>
+      <c r="H38" s="7"/>
+    </row>
+    <row r="39" spans="1:8">
       <c r="C39" s="10"/>
       <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
       <c r="F39" s="10"/>
       <c r="G39" s="10"/>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H39" s="10"/>
+    </row>
+    <row r="40" spans="1:8">
       <c r="C40" s="10"/>
       <c r="D40" s="10"/>
-      <c r="E40" s="10"/>
       <c r="F40" s="10"/>
-      <c r="G40" s="6"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G40" s="10"/>
+      <c r="H40" s="6"/>
+    </row>
+    <row r="41" spans="1:8">
       <c r="C41" s="10"/>
       <c r="D41" s="10"/>
-      <c r="E41" s="10"/>
       <c r="F41" s="10"/>
-      <c r="G41" s="6"/>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G41" s="10"/>
+      <c r="H41" s="6"/>
+    </row>
+    <row r="42" spans="1:8">
       <c r="C42" s="10"/>
       <c r="D42" s="10"/>
-      <c r="E42" s="10"/>
       <c r="F42" s="10"/>
-      <c r="G42" s="6"/>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G42" s="10"/>
+      <c r="H42" s="6"/>
+    </row>
+    <row r="43" spans="1:8">
       <c r="C43" s="10"/>
       <c r="D43" s="10"/>
-      <c r="E43" s="10"/>
       <c r="F43" s="10"/>
-      <c r="G43" s="6"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1911,19 +2069,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G44"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I44"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="48.140625" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" customWidth="1"/>
-    <col min="4" max="4" width="19.28515625" customWidth="1"/>
-    <col min="5" max="5" width="26.5703125" customWidth="1"/>
-    <col min="6" max="6" width="28" customWidth="1"/>
-    <col min="7" max="7" width="38.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="7" width="26.5703125" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
+    <col min="9" max="9" width="38.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="15.75">
       <c r="A1" s="2" t="s">
         <v>64</v>
       </c>
@@ -1936,17 +2095,23 @@
       <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="15.75">
       <c r="A2" s="6" t="s">
         <v>3</v>
       </c>
@@ -1955,13 +2120,17 @@
       </c>
       <c r="C2" s="9"/>
       <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
+      <c r="E2" s="14" t="s">
+        <v>281</v>
+      </c>
       <c r="F2" s="5"/>
-      <c r="G2" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="15.75">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
@@ -1970,13 +2139,17 @@
       </c>
       <c r="C3" s="9"/>
       <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
+      <c r="E3" s="15" t="s">
+        <v>280</v>
+      </c>
       <c r="F3" s="5"/>
-      <c r="G3" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="15.75">
       <c r="A4" s="6" t="s">
         <v>5</v>
       </c>
@@ -1985,43 +2158,55 @@
       </c>
       <c r="C4" s="9"/>
       <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
+      <c r="E4" s="14" t="s">
+        <v>276</v>
+      </c>
       <c r="F4" s="5"/>
-      <c r="G4" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="15.75">
       <c r="A5" s="6" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>159</v>
+        <v>284</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
+      <c r="E5" s="14" t="s">
+        <v>281</v>
+      </c>
       <c r="F5" s="5"/>
-      <c r="G5" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="15.75">
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C6" s="9"/>
       <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
+      <c r="E6" s="14" t="s">
+        <v>279</v>
+      </c>
       <c r="F6" s="5"/>
-      <c r="G6" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="15.75">
       <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
@@ -2030,478 +2215,606 @@
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
+      <c r="E7" s="14" t="s">
+        <v>277</v>
+      </c>
       <c r="F7" s="5"/>
-      <c r="G7" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="15.75">
       <c r="A8" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C8" s="9"/>
       <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+      <c r="E8" s="14" t="s">
+        <v>278</v>
+      </c>
       <c r="F8" s="5"/>
-      <c r="G8" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="15.75">
       <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C9" s="9"/>
       <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+      <c r="E9" s="14" t="s">
+        <v>278</v>
+      </c>
       <c r="F9" s="5"/>
-      <c r="G9" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="15.75">
       <c r="A10" s="6" t="s">
         <v>11</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C10" s="9"/>
       <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
+      <c r="E10" s="14" t="s">
+        <v>279</v>
+      </c>
       <c r="F10" s="5"/>
-      <c r="G10" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="15.75">
       <c r="A11" s="6" t="s">
         <v>12</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C11" s="9"/>
       <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
+      <c r="E11" s="14" t="s">
+        <v>278</v>
+      </c>
       <c r="F11" s="5"/>
-      <c r="G11" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="15.75">
       <c r="A12" s="6" t="s">
         <v>13</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C12" s="9"/>
       <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+      <c r="E12" s="15" t="s">
+        <v>280</v>
+      </c>
       <c r="F12" s="5"/>
-      <c r="G12" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="15.75">
       <c r="A13" s="6" t="s">
         <v>14</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C13" s="9"/>
       <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
+      <c r="E13" s="14" t="s">
+        <v>281</v>
+      </c>
       <c r="F13" s="5"/>
-      <c r="G13" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="15.75">
       <c r="A14" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C14" s="9"/>
       <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
+      <c r="E14" s="14" t="s">
+        <v>278</v>
+      </c>
       <c r="F14" s="5"/>
-      <c r="G14" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="15.75">
       <c r="A15" s="6" t="s">
         <v>16</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C15" s="9"/>
       <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
+      <c r="E15" s="15" t="s">
+        <v>280</v>
+      </c>
       <c r="F15" s="5"/>
-      <c r="G15" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="15.75">
       <c r="A16" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C16" s="9"/>
       <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
+      <c r="E16" s="14" t="s">
+        <v>277</v>
+      </c>
       <c r="F16" s="5"/>
-      <c r="G16" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="15.75">
       <c r="A17" s="6" t="s">
         <v>18</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
+      <c r="E17" s="14" t="s">
+        <v>277</v>
+      </c>
       <c r="F17" s="5"/>
-      <c r="G17" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+      <c r="I17" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="15.75">
       <c r="A18" s="6" t="s">
         <v>19</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C18" s="9"/>
       <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
+      <c r="E18" s="14" t="s">
+        <v>276</v>
+      </c>
       <c r="F18" s="5"/>
-      <c r="G18" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="15.75">
       <c r="A19" s="6" t="s">
         <v>20</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
+      <c r="E19" s="14" t="s">
+        <v>276</v>
+      </c>
       <c r="F19" s="5"/>
-      <c r="G19" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="15.75">
       <c r="A20" s="6" t="s">
         <v>21</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C20" s="9"/>
       <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
+      <c r="E20" s="14" t="s">
+        <v>276</v>
+      </c>
       <c r="F20" s="5"/>
-      <c r="G20" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="15.75">
       <c r="A21" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C21" s="9"/>
       <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
+      <c r="E21" s="14" t="s">
+        <v>281</v>
+      </c>
       <c r="F21" s="5"/>
-      <c r="G21" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="15.75">
       <c r="A22" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C22" s="9"/>
       <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
+      <c r="E22" s="14" t="s">
+        <v>276</v>
+      </c>
       <c r="F22" s="5"/>
-      <c r="G22" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+      <c r="I22" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="15.75">
       <c r="A23" s="6" t="s">
         <v>24</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C23" s="9"/>
       <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
+      <c r="E23" s="14" t="s">
+        <v>276</v>
+      </c>
       <c r="F23" s="5"/>
-      <c r="G23" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+      <c r="I23" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="15.75">
       <c r="A24" s="6" t="s">
         <v>25</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C24" s="9"/>
       <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
+      <c r="E24" s="14" t="s">
+        <v>277</v>
+      </c>
       <c r="F24" s="5"/>
-      <c r="G24" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+      <c r="I24" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="15.75">
       <c r="A25" s="6" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C25" s="9"/>
       <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
+      <c r="E25" s="14" t="s">
+        <v>279</v>
+      </c>
       <c r="F25" s="5"/>
-      <c r="G25" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="15.75">
       <c r="A26" s="6" t="s">
         <v>27</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C26" s="9"/>
       <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
+      <c r="E26" s="14" t="s">
+        <v>279</v>
+      </c>
       <c r="F26" s="5"/>
-      <c r="G26" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+      <c r="I26" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="15.75">
       <c r="A27" s="6" t="s">
         <v>28</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C27" s="9"/>
       <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
+      <c r="E27" s="14" t="s">
+        <v>278</v>
+      </c>
       <c r="F27" s="5"/>
-      <c r="G27" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+      <c r="I27" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="15.75">
       <c r="A28" s="6" t="s">
         <v>29</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C28" s="9"/>
       <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
+      <c r="E28" s="14" t="s">
+        <v>277</v>
+      </c>
       <c r="F28" s="5"/>
-      <c r="G28" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G28" s="5"/>
+      <c r="H28" s="5"/>
+      <c r="I28" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="15.75">
       <c r="A29" s="6" t="s">
         <v>30</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C29" s="9"/>
       <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
+      <c r="E29" s="14" t="s">
+        <v>277</v>
+      </c>
       <c r="F29" s="5"/>
-      <c r="G29" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="15.75">
       <c r="A30" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C30" s="9"/>
       <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
+      <c r="E30" s="14" t="s">
+        <v>281</v>
+      </c>
       <c r="F30" s="5"/>
-      <c r="G30" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G30" s="5"/>
+      <c r="H30" s="5"/>
+      <c r="I30" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="15.75">
       <c r="A31" s="6" t="s">
         <v>32</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C31" s="9"/>
       <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
+      <c r="E31" s="14" t="s">
+        <v>279</v>
+      </c>
       <c r="F31" s="5"/>
-      <c r="G31" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+      <c r="I31" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="15.75">
       <c r="A32" s="6" t="s">
         <v>33</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C32" s="9"/>
       <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
+      <c r="E32" s="14" t="s">
+        <v>281</v>
+      </c>
       <c r="F32" s="5"/>
-      <c r="G32" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+      <c r="I32" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="15.75">
       <c r="A33" s="6" t="s">
         <v>34</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C33" s="9"/>
       <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
+      <c r="E33" s="14" t="s">
+        <v>279</v>
+      </c>
       <c r="F33" s="5"/>
-      <c r="G33" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="15.75">
       <c r="A34" s="6" t="s">
         <v>145</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C34" s="9"/>
       <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
+      <c r="E34" s="14" t="s">
+        <v>277</v>
+      </c>
       <c r="F34" s="5"/>
-      <c r="G34" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+      <c r="I34" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="15.75">
       <c r="A35" s="6" t="s">
         <v>146</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C35" s="9"/>
       <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
+      <c r="E35" s="14" t="s">
+        <v>276</v>
+      </c>
       <c r="F35" s="5"/>
-      <c r="G35" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+      <c r="I35" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="15.75">
       <c r="A36" s="6" t="s">
         <v>147</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C36" s="9"/>
       <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
+      <c r="E36" s="14" t="s">
+        <v>278</v>
+      </c>
       <c r="F36" s="5"/>
-      <c r="G36" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G36" s="5"/>
+      <c r="H36" s="5"/>
+      <c r="I36" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="15.75">
       <c r="A37" s="6" t="s">
         <v>148</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C37" s="9"/>
       <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
+      <c r="E37" s="14" t="s">
+        <v>278</v>
+      </c>
       <c r="F37" s="5"/>
-      <c r="G37" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G37" s="5"/>
+      <c r="H37" s="5"/>
+      <c r="I37" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="15.75">
       <c r="A38" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B38" s="6" t="s">
         <v>190</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>191</v>
       </c>
       <c r="C38" s="9"/>
       <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
+      <c r="E38" s="14" t="s">
+        <v>281</v>
+      </c>
       <c r="F38" s="5"/>
-      <c r="G38" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G38" s="5"/>
+      <c r="H38" s="5"/>
+      <c r="I38" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="15.75">
       <c r="A39" s="6" t="s">
         <v>149</v>
       </c>
@@ -2510,85 +2823,109 @@
       </c>
       <c r="C39" s="9"/>
       <c r="D39" s="5"/>
-      <c r="E39" s="5"/>
+      <c r="E39" s="14" t="s">
+        <v>278</v>
+      </c>
       <c r="F39" s="5"/>
-      <c r="G39" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G39" s="5"/>
+      <c r="H39" s="5"/>
+      <c r="I39" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="15.75">
       <c r="A40" s="6" t="s">
         <v>151</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C40" s="9"/>
       <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
+      <c r="E40" s="14" t="s">
+        <v>278</v>
+      </c>
       <c r="F40" s="5"/>
-      <c r="G40" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G40" s="5"/>
+      <c r="H40" s="5"/>
+      <c r="I40" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="15.75">
       <c r="A41" s="6" t="s">
         <v>152</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C41" s="9"/>
       <c r="D41" s="5"/>
-      <c r="E41" s="5"/>
+      <c r="E41" s="15" t="s">
+        <v>280</v>
+      </c>
       <c r="F41" s="5"/>
-      <c r="G41" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G41" s="5"/>
+      <c r="H41" s="5"/>
+      <c r="I41" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="15.75">
       <c r="A42" s="6" t="s">
         <v>153</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C42" s="9"/>
       <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
+      <c r="E42" s="15" t="s">
+        <v>280</v>
+      </c>
       <c r="F42" s="5"/>
-      <c r="G42" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G42" s="5"/>
+      <c r="H42" s="5"/>
+      <c r="I42" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="15.75">
       <c r="A43" s="6" t="s">
         <v>154</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C43" s="9"/>
       <c r="D43" s="5"/>
-      <c r="E43" s="5"/>
+      <c r="E43" s="15" t="s">
+        <v>280</v>
+      </c>
       <c r="F43" s="5"/>
-      <c r="G43" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G43" s="5"/>
+      <c r="H43" s="5"/>
+      <c r="I43" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="15.75">
       <c r="A44" s="6" t="s">
         <v>155</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C44" s="9"/>
       <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
+      <c r="E44" s="14" t="s">
+        <v>279</v>
+      </c>
       <c r="F44" s="5"/>
-      <c r="G44" t="s">
-        <v>238</v>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5"/>
+      <c r="I44" t="s">
+        <v>237</v>
       </c>
     </row>
   </sheetData>

</xml_diff>